<commit_message>
chore: update news radar report 2026-07-25
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,32 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <color rgb="000000FF"/>
-      <u val="single"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -58,34 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9D9D9"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -453,65 +415,58 @@
   </sheetPr>
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>New Title</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Source Name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Publication Date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Hyperlink URL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cigna Projects $200 Million in Customer Medical Cost Savings Over Three Years Driven by Artificial Intelligence Deployment</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Cigna projects that its implementation of artificial intelligence technology will reduce customer medical costs by $200 million over three years. This multi-year cost containment initiative demonstrates how integrating technological tools into healthcare management can achieve significant expense reductions for clients.</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>The Mighty 790 KFGO</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Thu, 23 Jul 2026 11:30:17 GMT</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxQSHNmNmtTdmh5V0pGZlpUWEM2amdvT05NU2tDUkpVZ29uTWY5R1hMVHRDSFZuSUtJQkFEZDhjVXFqb0JWSFhCRTR6VzQ5VV83a2dPMVhOTzVEYzdBbVR4MURPWFJDcW1sWUlzNHRYc3NxZ09OTEhxRzl3NC1PMi12bktQSEZSbkZSQjFjRXdsRmY3RkhZVjYyOGZrNDJmMGszZU5QdmJpXzNoNHRRbTZEQ2t3MHBRUQ?oc=5</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Priority Health Partners With Color Health And Grail To Introduce New Cancer Support Programs</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Priority Health has partnered with Color Health and Grail to launch two innovative cancer support solutions aimed at improving early detection and navigation for patients. This initiative matters because cancer care represents one of the most significant cost drivers for self-funded employers and health plans, making early intervention critical for mitigating financial and clinical burdens. For business operations, this development highlights a growing trend toward integrated, tech-enabled oncology solutions that employers can leverage to improve employee health outcomes while better managing long-term specialty drug and healthcare expenditures.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MedCity News</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Fri, 24 Jul 2026 17:20:19 GMT</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxNV0pDcGlrUVNRTTBvZ1pkUENPWm1UejF0WXdkR1RmcFlLS3M5VUFOZlFkSnEyZlRKSlVJWkU0bW8xTURQeVYzSWFLM1kzM3A1YjhpUmhLbWdBZENtRTVGOFhvM0RtT0VZak9CSTVFSC1xZ0JZeWs4MW80ZFYxTFBTOWdCOGc2WEU2X3dvckN3TTFZcnA1WGdaNXFsUVJRV0ZkZXlkRmhtcEt0WW9O?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>